<commit_message>
Aug 8 24 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TS04AndTS07_ValidateERPSection.xlsx
+++ b/TestData/LV_TS04AndTS07_ValidateERPSection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E792E0A-1458-42C5-B3D8-3C28B80438B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5CC46C-2499-4A36-B333-6EC2C7752ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
changes 24 oct 24
</commit_message>
<xml_diff>
--- a/TestData/LV_TS04AndTS07_ValidateERPSection.xlsx
+++ b/TestData/LV_TS04AndTS07_ValidateERPSection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2156642-16CE-4886-A64B-9BEDDAA0E3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAB9D140-AC8B-4139-85C8-B24AD6E5D412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -293,9 +293,6 @@
     <t>Gemma Hardy</t>
   </si>
   <si>
-    <t>Indrajeet Singh</t>
-  </si>
-  <si>
     <t>Dimitri Drone</t>
   </si>
   <si>
@@ -351,6 +348,9 @@
   </si>
   <si>
     <t>No Restrictions</t>
+  </si>
+  <si>
+    <t>Ajay Nair</t>
   </si>
 </sst>
 </file>
@@ -727,18 +727,18 @@
         <v>80</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" t="s">
         <v>86</v>
       </c>
-      <c r="B2" t="s">
-        <v>87</v>
-      </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
         <v>69</v>
@@ -752,7 +752,7 @@
         <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
         <v>44</v>
@@ -760,13 +760,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" t="s">
         <v>84</v>
       </c>
-      <c r="B4" t="s">
-        <v>85</v>
-      </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
         <v>66</v>
@@ -784,12 +784,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -807,32 +807,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -976,7 +976,7 @@
         <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -997,7 +997,7 @@
         <v>8</v>
       </c>
       <c r="K2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L2" t="s">
         <v>52</v>
@@ -1068,10 +1068,10 @@
         <v>53</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -1092,7 +1092,7 @@
         <v>8</v>
       </c>
       <c r="K3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L3" t="s">
         <v>52</v>
@@ -1166,7 +1166,7 @@
         <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
@@ -1187,7 +1187,7 @@
         <v>8</v>
       </c>
       <c r="K4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L4" t="s">
         <v>52</v>
@@ -1241,7 +1241,7 @@
         <v>77</v>
       </c>
       <c r="AC4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AD4" t="s">
         <v>8</v>
@@ -1393,7 +1393,7 @@
         <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>56</v>
@@ -1404,7 +1404,7 @@
         <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
         <v>57</v>

</xml_diff>